<commit_message>
fix: correct factory names in supplier-factories.js
</commit_message>
<xml_diff>
--- a/assets/factory-supplier pair.xlsx
+++ b/assets/factory-supplier pair.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shoaib\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PACD\Github\Primark-Carton-Ordering-Supply-Integration-Platform\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26332292-8D7B-4D54-8A6C-537B9D3947EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17F66A1-0103-42E0-B0D9-92C4A803E512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{928ABD3F-8EBF-4272-A8D8-EFC323556158}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{928ABD3F-8EBF-4272-A8D8-EFC323556158}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>SNQS GLOBAL TEXTILES FZE</t>
   </si>
   <si>
-    <t>Alim Knit Ltd</t>
-  </si>
-  <si>
     <t>Fame Apparels Ltd</t>
   </si>
   <si>
@@ -365,9 +362,6 @@
     <t>Soorty Textiles BD Limited PJT</t>
   </si>
   <si>
-    <t>SIMPLE APPROACH LIMTED</t>
-  </si>
-  <si>
     <t>ATS Apparels Ltd</t>
   </si>
   <si>
@@ -434,9 +428,6 @@
     <t>Good Bags And Accessories Limited</t>
   </si>
   <si>
-    <t>KAIXI FASHION (HK) CO.LTD</t>
-  </si>
-  <si>
     <t>Kaixi Fashion Bangladesh Co Ltd</t>
   </si>
   <si>
@@ -461,9 +452,6 @@
     <t>ECHO SOURCING LTD ROW</t>
   </si>
   <si>
-    <t>Far East Knitting &amp; Dyeing Industries Ltd PJT (115</t>
-  </si>
-  <si>
     <t>Echoknits Ltd</t>
   </si>
   <si>
@@ -497,9 +485,6 @@
     <t>PADMA TEXTILES LTD</t>
   </si>
   <si>
-    <t>Saturn Textile Limited</t>
-  </si>
-  <si>
     <t>Aspire Garments Ltd PJT</t>
   </si>
   <si>
@@ -515,9 +500,6 @@
     <t>ZAMIRA FASHION LIMITED</t>
   </si>
   <si>
-    <t>Dhaka Garments &amp; Washing Ltd PKA HAMS Washing &amp; Dy</t>
-  </si>
-  <si>
     <t>NOVEL HURRICANE KNIT GARMENTS LTD</t>
   </si>
   <si>
@@ -632,9 +614,6 @@
     <t>Colors &amp; Stitches Limited</t>
   </si>
   <si>
-    <t>Comfit Composite Knit Ltd PKA Comfit Lingerie Limi</t>
-  </si>
-  <si>
     <t>APS Apparels Limited</t>
   </si>
   <si>
@@ -651,6 +630,27 @@
   </si>
   <si>
     <t>Denim Asia Ltd PJT</t>
+  </si>
+  <si>
+    <t>Alim Knit (BD) Ltd</t>
+  </si>
+  <si>
+    <t>SIMPLE APPROACH LIMITED</t>
+  </si>
+  <si>
+    <t>Far East Knitting &amp; Dyeing Industries Ltd PJT</t>
+  </si>
+  <si>
+    <t>Saturn Textiles Limited</t>
+  </si>
+  <si>
+    <t>Dhaka Garments &amp; Washing Ltd</t>
+  </si>
+  <si>
+    <t>Comfit Composite Knit Ltd PKA Comfit Lingerie Limited</t>
+  </si>
+  <si>
+    <t>KAIXI FASHION (HK) CO. LTD</t>
   </si>
 </sst>
 </file>
@@ -1055,15 +1055,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B672399-E02E-4772-BA70-1094F7C80E3E}">
   <dimension ref="A1:D180"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>52745</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>52745</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>53438</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>53438</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>53438</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>54552</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>54552</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>54579</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>54579</v>
       </c>
@@ -1203,7 +1203,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>55790</v>
       </c>
@@ -1214,10 +1214,10 @@
         <v>20331</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>55790</v>
       </c>
@@ -1228,645 +1228,645 @@
         <v>25042</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>56331</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="3">
         <v>15187</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>56331</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" s="2">
         <v>15391</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>56331</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" s="3">
         <v>20979</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>56331</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="2">
         <v>26055</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>59407</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C17" s="3">
         <v>14279</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>59407</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="2">
         <v>17803</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>59407</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" s="3">
         <v>18938</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>59407</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2">
         <v>25383</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>59407</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C21" s="3">
         <v>26006</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>59407</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C22" s="2">
         <v>26425</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>59544</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" s="3">
         <v>11266</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>59544</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" s="2">
         <v>26005</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>59544</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25" s="3">
         <v>26451</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>60354</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C26" s="2">
         <v>25133</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>61116</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" s="3">
         <v>21750</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>61116</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28" s="2">
         <v>22846</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>61116</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29" s="3">
         <v>25218</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>61116</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30" s="2">
         <v>26055</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>61116</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="3">
         <v>26764</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>61116</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32" s="2">
         <v>27725</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>61301</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C33" s="3">
         <v>11583</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>64891</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C34" s="2">
         <v>15187</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>64951</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C35" s="3">
         <v>11583</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>64951</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C36" s="2">
         <v>14512</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>65163</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C37" s="3">
         <v>20421</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>65625</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C38" s="2">
         <v>16401</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>65863</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C39" s="3">
         <v>11583</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>66025</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C40" s="2">
         <v>25278</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>66440</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C41" s="3">
         <v>19424</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>66440</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C42" s="2">
         <v>23385</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>66440</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C43" s="3">
         <v>24272</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>66440</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C44" s="2">
         <v>24650</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>66440</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C45" s="3">
         <v>25236</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>66747</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C46" s="2">
         <v>16401</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>67604</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C47" s="3">
         <v>15735</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>67912</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C48" s="2">
         <v>26451</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>68683</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C49" s="3">
         <v>26447</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>68740</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C50" s="2">
         <v>24374</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>72380</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C51" s="3">
         <v>11277</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>72380</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C52" s="2">
         <v>24442</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>73151</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C53" s="3">
         <v>11583</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>73353</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C54" s="2">
         <v>19394</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>73353</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C55" s="3">
         <v>27650</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>73768</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C56" s="2">
         <v>27586</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>73968</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C57" s="3">
         <v>11277</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>73968</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C58" s="2">
         <v>17443</v>
@@ -1875,12 +1875,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>73975</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C59" s="3">
         <v>17443</v>
@@ -1889,54 +1889,54 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>76707</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C60" s="2">
         <v>14512</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>80044</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C61" s="3">
         <v>23445</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>80057</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C62" s="2">
         <v>20096</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>80057</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C63" s="3">
         <v>22933</v>
@@ -1945,670 +1945,670 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>80057</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C64" s="2">
         <v>25086</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>80057</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C65" s="3">
         <v>27826</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>80068</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C66" s="2">
         <v>18757</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>80068</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C67" s="3">
         <v>23925</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>80068</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C68" s="2">
         <v>23926</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>80068</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C69" s="3">
         <v>24407</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>80074</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C70" s="2">
         <v>14100</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>80083</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C71" s="3">
         <v>18001</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>80083</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C72" s="2">
         <v>21164</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>80171</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C73" s="3">
         <v>15173</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>80172</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C74" s="2">
         <v>22846</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>80195</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C75" s="3">
         <v>10077</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>80195</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C76" s="2">
         <v>10900</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>80222</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C77" s="3">
         <v>27672</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>80282</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C78" s="2">
         <v>20079</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>80306</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C79" s="3">
         <v>11121</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>80306</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C80" s="2">
         <v>13809</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80306</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C81" s="3">
         <v>15379</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>80306</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C82" s="2">
         <v>16534</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>80306</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C83" s="3">
         <v>17149</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>80306</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C84" s="2">
         <v>23378</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>80306</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C85" s="3">
         <v>23489</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>80306</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C86" s="2">
         <v>23926</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>80306</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C87" s="3">
         <v>24650</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
         <v>80306</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C88" s="2">
         <v>25399</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>80306</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C89" s="3">
         <v>25406</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
         <v>80306</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C90" s="2">
         <v>25547</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>80306</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C91" s="3">
         <v>25787</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
         <v>80306</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C92" s="2">
         <v>25968</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>80306</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C93" s="3">
         <v>25990</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
         <v>80306</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C94" s="2">
         <v>26306</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>80306</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C95" s="3">
         <v>26695</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
         <v>80306</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>108</v>
+        <v>198</v>
       </c>
       <c r="C96" s="2">
         <v>28381</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>80486</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C97" s="3">
         <v>24407</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
         <v>80486</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C98" s="2">
         <v>24634</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>80486</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C99" s="3">
         <v>24718</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
         <v>80486</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C100" s="2">
         <v>25438</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>80539</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C101" s="3">
         <v>27410</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
         <v>80734</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>131</v>
+        <v>203</v>
       </c>
       <c r="C102" s="2">
         <v>26163</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>80734</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>131</v>
+        <v>203</v>
       </c>
       <c r="C103" s="3">
         <v>27618</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
         <v>81107</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C104" s="2">
         <v>11277</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>81107</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C105" s="3">
         <v>24777</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
         <v>81107</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C106" s="2">
         <v>26088</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>81813</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C107" s="3">
         <v>19683</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
         <v>83001</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C108" s="2">
         <v>11277</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>83001</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C109" s="3">
         <v>11583</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
         <v>83001</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C110" s="2">
         <v>11584</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>83001</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C111" s="3">
         <v>17443</v>
@@ -2617,194 +2617,194 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
         <v>83001</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C112" s="2">
         <v>26559</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>83343</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C113" s="3">
         <v>11583</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
         <v>83343</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C114" s="2">
         <v>14512</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>83343</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C115" s="3">
         <v>18938</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
         <v>83393</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C116" s="2">
         <v>14542</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>83393</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C117" s="3">
         <v>20614</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
         <v>83468</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C118" s="2">
         <v>11266</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>83489</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C119" s="3">
         <v>15187</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
         <v>83515</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C120" s="2">
         <v>12048</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>83756</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C121" s="3">
         <v>15391</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
         <v>83760</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C122" s="2">
         <v>11277</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>83760</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C123" s="3">
         <v>14512</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
         <v>83760</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C124" s="2">
         <v>18234</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>83760</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C125" s="3">
         <v>20017</v>
@@ -2813,774 +2813,774 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
         <v>83760</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C126" s="2">
         <v>24040</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>83760</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C127" s="3">
         <v>25218</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
         <v>83760</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C128" s="2">
         <v>26387</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
         <v>83760</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C129" s="3">
         <v>27035</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
         <v>83760</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C130" s="2">
         <v>27649</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>83765</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C131" s="3">
         <v>22775</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>83804</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C132" s="2">
         <v>14482</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
         <v>83804</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C133" s="3">
         <v>18469</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
         <v>83804</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C134" s="2">
         <v>25086</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>83810</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C135" s="3">
         <v>14059</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
         <v>83810</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C136" s="2">
         <v>17803</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>83810</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C137" s="3">
         <v>18750</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
         <v>83810</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C138" s="2">
         <v>19424</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>83810</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C139" s="3">
         <v>25696</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
         <v>83834</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C140" s="2">
         <v>20015</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="3">
         <v>83834</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C141" s="3">
         <v>22806</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
         <v>83942</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C142" s="2">
         <v>19151</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="3">
         <v>83942</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C143" s="3">
         <v>20227</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
         <v>83942</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C144" s="2">
         <v>23609</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="3">
         <v>83942</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C145" s="3">
         <v>25905</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
         <v>83942</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C146" s="2">
         <v>26569</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="3">
         <v>83956</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C147" s="3">
         <v>11277</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
         <v>83956</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C148" s="2">
         <v>14482</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="3">
         <v>83956</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C149" s="3">
         <v>24442</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
         <v>83967</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C150" s="2">
         <v>19681</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="3">
         <v>83967</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C151" s="3">
         <v>20517</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
         <v>83967</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C152" s="2">
         <v>21111</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="3">
         <v>83967</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C153" s="3">
         <v>22400</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
         <v>83967</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C154" s="2">
         <v>22585</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="3">
         <v>83967</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C155" s="3">
         <v>22846</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
         <v>83967</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C156" s="2">
         <v>23445</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
         <v>83967</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C157" s="3">
         <v>23817</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
         <v>83967</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C158" s="2">
         <v>27586</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="3">
         <v>83967</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C159" s="3">
         <v>27798</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
         <v>83998</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C160" s="2">
         <v>15378</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="3">
         <v>83998</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C161" s="3">
         <v>18763</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
         <v>83998</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C162" s="2">
         <v>24250</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="3">
         <v>84016</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C163" s="3">
         <v>11277</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
         <v>84081</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C164" s="2">
         <v>11277</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="3">
         <v>84081</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C165" s="3">
         <v>11583</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
         <v>84081</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C166" s="2">
         <v>18469</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>84130</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C167" s="3">
         <v>20096</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
         <v>84177</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C168" s="2">
         <v>18926</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="3">
         <v>84177</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C169" s="3">
         <v>18983</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>84177</v>
       </c>
       <c r="B170" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C170">
         <v>20147</v>
       </c>
       <c r="D170" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>84177</v>
       </c>
       <c r="B171" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C171">
         <v>20159</v>
       </c>
       <c r="D171" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>84177</v>
       </c>
       <c r="B172" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C172">
         <v>24442</v>
       </c>
       <c r="D172" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>84177</v>
       </c>
       <c r="B173" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C173">
         <v>24447</v>
       </c>
       <c r="D173" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>84177</v>
       </c>
       <c r="B174" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C174">
         <v>24448</v>
       </c>
       <c r="D174" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>84177</v>
       </c>
       <c r="B175" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C175">
         <v>26018</v>
       </c>
       <c r="D175" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>84177</v>
       </c>
       <c r="B176" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C176">
         <v>26150</v>
       </c>
       <c r="D176" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>84177</v>
       </c>
       <c r="B177" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="C177">
         <v>26293</v>
       </c>
       <c r="D177" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>84230</v>
       </c>
       <c r="B178" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C178">
         <v>27826</v>
       </c>
       <c r="D178" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>84257</v>
       </c>
       <c r="B179" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="C179">
         <v>23908</v>
       </c>
       <c r="D179" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>84257</v>
       </c>
       <c r="B180" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="C180">
         <v>24040</v>
       </c>
       <c r="D180" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update factory name from Mohammadi Group Limited to MG Niche Flair Limited Unit 2
</commit_message>
<xml_diff>
--- a/assets/factory-supplier pair.xlsx
+++ b/assets/factory-supplier pair.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PACD\Github\Primark-Carton-Ordering-Supply-Integration-Platform\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17F66A1-0103-42E0-B0D9-92C4A803E512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DEE727D-5A39-47C4-ABBB-4BA6CFC75CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{928ABD3F-8EBF-4272-A8D8-EFC323556158}"/>
   </bookViews>
@@ -158,9 +158,6 @@
     <t>Glory Fashion Wear Ltd</t>
   </si>
   <si>
-    <t>Mohammadi Group Limited</t>
-  </si>
-  <si>
     <t>Fortis Garments Limited</t>
   </si>
   <si>
@@ -651,6 +648,9 @@
   </si>
   <si>
     <t>KAIXI FASHION (HK) CO. LTD</t>
+  </si>
+  <si>
+    <t>MG Niche Flair Limited Unit 2</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1214,7 @@
         <v>20331</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1452,7 +1452,7 @@
         <v>22846</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -1466,7 +1466,7 @@
         <v>25218</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1494,7 +1494,7 @@
         <v>26764</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1508,7 +1508,7 @@
         <v>27725</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1516,13 +1516,13 @@
         <v>61301</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="3">
         <v>11583</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1530,7 +1530,7 @@
         <v>64891</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C34" s="2">
         <v>15187</v>
@@ -1544,13 +1544,13 @@
         <v>64951</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C35" s="3">
         <v>11583</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1558,13 +1558,13 @@
         <v>64951</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C36" s="2">
         <v>14512</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
@@ -1572,13 +1572,13 @@
         <v>65163</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C37" s="3">
         <v>20421</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -1586,13 +1586,13 @@
         <v>65625</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C38" s="2">
         <v>16401</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
@@ -1600,13 +1600,13 @@
         <v>65863</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C39" s="3">
         <v>11583</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
@@ -1614,13 +1614,13 @@
         <v>66025</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C40" s="2">
         <v>25278</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
@@ -1628,13 +1628,13 @@
         <v>66440</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C41" s="3">
         <v>19424</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
@@ -1642,13 +1642,13 @@
         <v>66440</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C42" s="2">
         <v>23385</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
@@ -1656,13 +1656,13 @@
         <v>66440</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C43" s="3">
         <v>24272</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
@@ -1670,13 +1670,13 @@
         <v>66440</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C44" s="2">
         <v>24650</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1684,13 +1684,13 @@
         <v>66440</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C45" s="3">
         <v>25236</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
@@ -1698,13 +1698,13 @@
         <v>66747</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C46" s="2">
         <v>16401</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1712,13 +1712,13 @@
         <v>67604</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C47" s="3">
         <v>15735</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -1726,7 +1726,7 @@
         <v>67912</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C48" s="2">
         <v>26451</v>
@@ -1740,13 +1740,13 @@
         <v>68683</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C49" s="3">
         <v>26447</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -1754,13 +1754,13 @@
         <v>68740</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C50" s="2">
         <v>24374</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -1768,13 +1768,13 @@
         <v>72380</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C51" s="3">
         <v>11277</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -1782,13 +1782,13 @@
         <v>72380</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C52" s="2">
         <v>24442</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -1796,13 +1796,13 @@
         <v>73151</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C53" s="3">
         <v>11583</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -1810,13 +1810,13 @@
         <v>73353</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C54" s="2">
         <v>19394</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -1824,13 +1824,13 @@
         <v>73353</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C55" s="3">
         <v>27650</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -1838,13 +1838,13 @@
         <v>73768</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C56" s="2">
         <v>27586</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1852,13 +1852,13 @@
         <v>73968</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C57" s="3">
         <v>11277</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -1866,7 +1866,7 @@
         <v>73968</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C58" s="2">
         <v>17443</v>
@@ -1880,7 +1880,7 @@
         <v>73975</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C59" s="3">
         <v>17443</v>
@@ -1894,13 +1894,13 @@
         <v>76707</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C60" s="2">
         <v>14512</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -1908,13 +1908,13 @@
         <v>80044</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C61" s="3">
         <v>23445</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1922,13 +1922,13 @@
         <v>80057</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C62" s="2">
         <v>20096</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
@@ -1936,7 +1936,7 @@
         <v>80057</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C63" s="3">
         <v>22933</v>
@@ -1950,13 +1950,13 @@
         <v>80057</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C64" s="2">
         <v>25086</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
@@ -1964,13 +1964,13 @@
         <v>80057</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C65" s="3">
         <v>27826</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
@@ -1978,13 +1978,13 @@
         <v>80068</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C66" s="2">
         <v>18757</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
@@ -1992,13 +1992,13 @@
         <v>80068</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C67" s="3">
         <v>23925</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
@@ -2006,13 +2006,13 @@
         <v>80068</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C68" s="2">
         <v>23926</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
@@ -2020,13 +2020,13 @@
         <v>80068</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C69" s="3">
         <v>24407</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
@@ -2034,13 +2034,13 @@
         <v>80074</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C70" s="2">
         <v>14100</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
@@ -2048,13 +2048,13 @@
         <v>80083</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C71" s="3">
         <v>18001</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
@@ -2062,13 +2062,13 @@
         <v>80083</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C72" s="2">
         <v>21164</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
@@ -2076,13 +2076,13 @@
         <v>80171</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C73" s="3">
         <v>15173</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2090,13 +2090,13 @@
         <v>80172</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C74" s="2">
         <v>22846</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
@@ -2104,13 +2104,13 @@
         <v>80195</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C75" s="3">
         <v>10077</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
@@ -2118,13 +2118,13 @@
         <v>80195</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C76" s="2">
         <v>10900</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
@@ -2132,13 +2132,13 @@
         <v>80222</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C77" s="3">
         <v>27672</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
@@ -2146,13 +2146,13 @@
         <v>80282</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C78" s="2">
         <v>20079</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
@@ -2160,13 +2160,13 @@
         <v>80306</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C79" s="3">
         <v>11121</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -2174,13 +2174,13 @@
         <v>80306</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C80" s="2">
         <v>13809</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
@@ -2188,13 +2188,13 @@
         <v>80306</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C81" s="3">
         <v>15379</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
@@ -2202,13 +2202,13 @@
         <v>80306</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C82" s="2">
         <v>16534</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
@@ -2216,13 +2216,13 @@
         <v>80306</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C83" s="3">
         <v>17149</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
@@ -2230,13 +2230,13 @@
         <v>80306</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C84" s="2">
         <v>23378</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
@@ -2244,13 +2244,13 @@
         <v>80306</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C85" s="3">
         <v>23489</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
@@ -2258,13 +2258,13 @@
         <v>80306</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C86" s="2">
         <v>23926</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
@@ -2272,13 +2272,13 @@
         <v>80306</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C87" s="3">
         <v>24650</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -2286,13 +2286,13 @@
         <v>80306</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C88" s="2">
         <v>25399</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
@@ -2300,13 +2300,13 @@
         <v>80306</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C89" s="3">
         <v>25406</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
@@ -2314,13 +2314,13 @@
         <v>80306</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C90" s="2">
         <v>25547</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
@@ -2328,13 +2328,13 @@
         <v>80306</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C91" s="3">
         <v>25787</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
@@ -2342,13 +2342,13 @@
         <v>80306</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C92" s="2">
         <v>25968</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
@@ -2356,13 +2356,13 @@
         <v>80306</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C93" s="3">
         <v>25990</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
@@ -2370,13 +2370,13 @@
         <v>80306</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C94" s="2">
         <v>26306</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
@@ -2384,13 +2384,13 @@
         <v>80306</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C95" s="3">
         <v>26695</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
@@ -2398,13 +2398,13 @@
         <v>80306</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C96" s="2">
         <v>28381</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
@@ -2412,13 +2412,13 @@
         <v>80486</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C97" s="3">
         <v>24407</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -2426,13 +2426,13 @@
         <v>80486</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C98" s="2">
         <v>24634</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
@@ -2440,13 +2440,13 @@
         <v>80486</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C99" s="3">
         <v>24718</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2454,13 +2454,13 @@
         <v>80486</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C100" s="2">
         <v>25438</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
@@ -2468,13 +2468,13 @@
         <v>80539</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C101" s="3">
         <v>27410</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -2482,13 +2482,13 @@
         <v>80734</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C102" s="2">
         <v>26163</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
@@ -2496,13 +2496,13 @@
         <v>80734</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C103" s="3">
         <v>27618</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -2510,13 +2510,13 @@
         <v>81107</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C104" s="2">
         <v>11277</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2524,13 +2524,13 @@
         <v>81107</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C105" s="3">
         <v>24777</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -2538,13 +2538,13 @@
         <v>81107</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C106" s="2">
         <v>26088</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
@@ -2552,13 +2552,13 @@
         <v>81813</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C107" s="3">
         <v>19683</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
@@ -2566,13 +2566,13 @@
         <v>83001</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C108" s="2">
         <v>11277</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
@@ -2580,13 +2580,13 @@
         <v>83001</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C109" s="3">
         <v>11583</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -2594,13 +2594,13 @@
         <v>83001</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C110" s="2">
         <v>11584</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -2608,7 +2608,7 @@
         <v>83001</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C111" s="3">
         <v>17443</v>
@@ -2622,13 +2622,13 @@
         <v>83001</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C112" s="2">
         <v>26559</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -2636,13 +2636,13 @@
         <v>83343</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C113" s="3">
         <v>11583</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.25">
@@ -2650,13 +2650,13 @@
         <v>83343</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C114" s="2">
         <v>14512</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
@@ -2664,7 +2664,7 @@
         <v>83343</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C115" s="3">
         <v>18938</v>
@@ -2678,13 +2678,13 @@
         <v>83393</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C116" s="2">
         <v>14542</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
@@ -2692,13 +2692,13 @@
         <v>83393</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C117" s="3">
         <v>20614</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
@@ -2706,7 +2706,7 @@
         <v>83468</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C118" s="2">
         <v>11266</v>
@@ -2720,7 +2720,7 @@
         <v>83489</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C119" s="3">
         <v>15187</v>
@@ -2734,13 +2734,13 @@
         <v>83515</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C120" s="2">
         <v>12048</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
@@ -2748,7 +2748,7 @@
         <v>83756</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C121" s="3">
         <v>15391</v>
@@ -2762,13 +2762,13 @@
         <v>83760</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C122" s="2">
         <v>11277</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
@@ -2776,13 +2776,13 @@
         <v>83760</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C123" s="3">
         <v>14512</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
@@ -2790,13 +2790,13 @@
         <v>83760</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C124" s="2">
         <v>18234</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
@@ -2804,7 +2804,7 @@
         <v>83760</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C125" s="3">
         <v>20017</v>
@@ -2818,13 +2818,13 @@
         <v>83760</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C126" s="2">
         <v>24040</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
@@ -2832,13 +2832,13 @@
         <v>83760</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C127" s="3">
         <v>25218</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
@@ -2846,13 +2846,13 @@
         <v>83760</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C128" s="2">
         <v>26387</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
@@ -2860,13 +2860,13 @@
         <v>83760</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C129" s="3">
         <v>27035</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.25">
@@ -2874,13 +2874,13 @@
         <v>83760</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C130" s="2">
         <v>27649</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.25">
@@ -2888,13 +2888,13 @@
         <v>83765</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C131" s="3">
         <v>22775</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
@@ -2902,13 +2902,13 @@
         <v>83804</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C132" s="2">
         <v>14482</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.25">
@@ -2916,13 +2916,13 @@
         <v>83804</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C133" s="3">
         <v>18469</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.25">
@@ -2930,13 +2930,13 @@
         <v>83804</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C134" s="2">
         <v>25086</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.25">
@@ -2944,13 +2944,13 @@
         <v>83810</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C135" s="3">
         <v>14059</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
@@ -2958,7 +2958,7 @@
         <v>83810</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C136" s="2">
         <v>17803</v>
@@ -2972,13 +2972,13 @@
         <v>83810</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C137" s="3">
         <v>18750</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
@@ -2986,13 +2986,13 @@
         <v>83810</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C138" s="2">
         <v>19424</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.25">
@@ -3000,13 +3000,13 @@
         <v>83810</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C139" s="3">
         <v>25696</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.25">
@@ -3014,13 +3014,13 @@
         <v>83834</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C140" s="2">
         <v>20015</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.25">
@@ -3028,13 +3028,13 @@
         <v>83834</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C141" s="3">
         <v>22806</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
@@ -3042,13 +3042,13 @@
         <v>83942</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C142" s="2">
         <v>19151</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
@@ -3056,13 +3056,13 @@
         <v>83942</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C143" s="3">
         <v>20227</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
@@ -3070,13 +3070,13 @@
         <v>83942</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C144" s="2">
         <v>23609</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.25">
@@ -3084,13 +3084,13 @@
         <v>83942</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C145" s="3">
         <v>25905</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.25">
@@ -3098,13 +3098,13 @@
         <v>83942</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C146" s="2">
         <v>26569</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
@@ -3112,13 +3112,13 @@
         <v>83956</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C147" s="3">
         <v>11277</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.25">
@@ -3126,13 +3126,13 @@
         <v>83956</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C148" s="2">
         <v>14482</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.25">
@@ -3140,13 +3140,13 @@
         <v>83956</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C149" s="3">
         <v>24442</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
@@ -3154,13 +3154,13 @@
         <v>83967</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C150" s="2">
         <v>19681</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
@@ -3168,13 +3168,13 @@
         <v>83967</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C151" s="3">
         <v>20517</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.25">
@@ -3182,13 +3182,13 @@
         <v>83967</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C152" s="2">
         <v>21111</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.25">
@@ -3196,13 +3196,13 @@
         <v>83967</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C153" s="3">
         <v>22400</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.25">
@@ -3210,13 +3210,13 @@
         <v>83967</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C154" s="2">
         <v>22585</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.25">
@@ -3224,13 +3224,13 @@
         <v>83967</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C155" s="3">
         <v>22846</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>39</v>
+        <v>203</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.25">
@@ -3238,13 +3238,13 @@
         <v>83967</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C156" s="2">
         <v>23445</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.25">
@@ -3252,13 +3252,13 @@
         <v>83967</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C157" s="3">
         <v>23817</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.25">
@@ -3266,13 +3266,13 @@
         <v>83967</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C158" s="2">
         <v>27586</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.25">
@@ -3280,13 +3280,13 @@
         <v>83967</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C159" s="3">
         <v>27798</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.25">
@@ -3294,13 +3294,13 @@
         <v>83998</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C160" s="2">
         <v>15378</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
@@ -3308,13 +3308,13 @@
         <v>83998</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C161" s="3">
         <v>18763</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
@@ -3322,13 +3322,13 @@
         <v>83998</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C162" s="2">
         <v>24250</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
@@ -3336,13 +3336,13 @@
         <v>84016</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C163" s="3">
         <v>11277</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.25">
@@ -3350,13 +3350,13 @@
         <v>84081</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C164" s="2">
         <v>11277</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.25">
@@ -3364,13 +3364,13 @@
         <v>84081</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C165" s="3">
         <v>11583</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.25">
@@ -3378,13 +3378,13 @@
         <v>84081</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C166" s="2">
         <v>18469</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.25">
@@ -3392,13 +3392,13 @@
         <v>84130</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C167" s="3">
         <v>20096</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.25">
@@ -3406,13 +3406,13 @@
         <v>84177</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C168" s="2">
         <v>18926</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.25">
@@ -3420,13 +3420,13 @@
         <v>84177</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C169" s="3">
         <v>18983</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.25">
@@ -3434,13 +3434,13 @@
         <v>84177</v>
       </c>
       <c r="B170" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C170">
         <v>20147</v>
       </c>
       <c r="D170" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.25">
@@ -3448,13 +3448,13 @@
         <v>84177</v>
       </c>
       <c r="B171" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C171">
         <v>20159</v>
       </c>
       <c r="D171" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
@@ -3462,13 +3462,13 @@
         <v>84177</v>
       </c>
       <c r="B172" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C172">
         <v>24442</v>
       </c>
       <c r="D172" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.25">
@@ -3476,13 +3476,13 @@
         <v>84177</v>
       </c>
       <c r="B173" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C173">
         <v>24447</v>
       </c>
       <c r="D173" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
@@ -3490,13 +3490,13 @@
         <v>84177</v>
       </c>
       <c r="B174" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C174">
         <v>24448</v>
       </c>
       <c r="D174" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.25">
@@ -3504,13 +3504,13 @@
         <v>84177</v>
       </c>
       <c r="B175" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C175">
         <v>26018</v>
       </c>
       <c r="D175" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.25">
@@ -3518,13 +3518,13 @@
         <v>84177</v>
       </c>
       <c r="B176" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C176">
         <v>26150</v>
       </c>
       <c r="D176" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.25">
@@ -3532,13 +3532,13 @@
         <v>84177</v>
       </c>
       <c r="B177" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C177">
         <v>26293</v>
       </c>
       <c r="D177" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.25">
@@ -3546,13 +3546,13 @@
         <v>84230</v>
       </c>
       <c r="B178" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C178">
         <v>27826</v>
       </c>
       <c r="D178" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.25">
@@ -3560,13 +3560,13 @@
         <v>84257</v>
       </c>
       <c r="B179" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C179">
         <v>23908</v>
       </c>
       <c r="D179" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.25">
@@ -3574,13 +3574,13 @@
         <v>84257</v>
       </c>
       <c r="B180" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C180">
         <v>24040</v>
       </c>
       <c r="D180" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>